<commit_message>
Made another dent in firmware
</commit_message>
<xml_diff>
--- a/hardware/Clay Counter BOM - Rev4.0.xlsx
+++ b/hardware/Clay Counter BOM - Rev4.0.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jaxon\Documents\001_Projects\Clay Counter\hardware\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EB70B17-E14B-409B-99D6-D464239BD3FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6E28FCF-F2B4-47BD-A75F-90232ECE7279}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="15585" xr2:uid="{FBC6EBE0-28E6-48B1-ABE0-6D26B9367613}"/>
+    <workbookView xWindow="0" yWindow="1500" windowWidth="23190" windowHeight="10920" xr2:uid="{FBC6EBE0-28E6-48B1-ABE0-6D26B9367613}"/>
   </bookViews>
   <sheets>
     <sheet name="Clay Counter BOM - Rev4.0" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="40">
   <si>
     <t>RefDes</t>
   </si>
@@ -137,6 +137,9 @@
   </si>
   <si>
     <t>Unikeyic</t>
+  </si>
+  <si>
+    <t>Universal Solder</t>
   </si>
 </sst>
 </file>
@@ -1145,7 +1148,7 @@
         <v>1</v>
       </c>
       <c r="F3" s="13" t="s">
-        <v>18</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="1:6" s="10" customFormat="1" x14ac:dyDescent="0.25">

</xml_diff>